<commit_message>
feat(master): include jenis/sites sheets in alats XLSX template
</commit_message>
<xml_diff>
--- a/web/public/templates/alats-template.xlsx
+++ b/web/public/templates/alats-template.xlsx
@@ -4,6 +4,8 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="alats-template" sheetId="1" r:id="rId1"/>
+    <sheet name="jenis-template" sheetId="2" r:id="rId2"/>
+    <sheet name="sites-template" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -456,4 +458,103 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nama</v>
+      </c>
+      <c r="C1" t="str">
+        <v>description</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Generator</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Diesel generator set</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Pump</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Water pump / centrifugal</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Compressor</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Air compressor</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>code</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Site A</v>
+      </c>
+      <c r="C2" t="str">
+        <v>SITE-A</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>20</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Site B</v>
+      </c>
+      <c r="C3" t="str">
+        <v>SITE-B</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>